<commit_message>
YHAAO-18682 zkb fe excel到处报表优化 web开发
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/zkb/partOrder/excel/APM_ZKB_PartOrder_Exp_Template.xlsx
+++ b/src/src/main/webapp/portal/zkb/partOrder/excel/APM_ZKB_PartOrder_Exp_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Intellij Idea\codes\hc-apm-web\src\src\main\webapp\portal\zkb\partOrder\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\hc-apm-web\src\src\main\webapp\portal\zkb\partOrder\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09422F32-063F-468B-A0CA-261C8FA01A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF6F03C-8523-471A-AA61-2CF74F31BF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="358" activeTab="4" xr2:uid="{DFA98752-8825-45D1-95EF-55416474EBE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="358" xr2:uid="{DFA98752-8825-45D1-95EF-55416474EBE9}"/>
   </bookViews>
   <sheets>
     <sheet name="维修工单" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="66">
   <si>
     <t>区域</t>
   </si>
@@ -66,6 +66,8 @@
         <sz val="13.5"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>SN(序列号)</t>
     </r>
@@ -79,6 +81,8 @@
         <sz val="13.5"/>
         <color theme="1"/>
         <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
       </rPr>
       <t>注（说明是否DOA或者Short life）</t>
     </r>
@@ -250,17 +254,21 @@
   </si>
   <si>
     <t>是否需要Dongle</t>
+  </si>
+  <si>
+    <t>下单时间</t>
+    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -268,21 +276,36 @@
       <sz val="12"/>
       <color rgb="FF172B4D"/>
       <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="13.5"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -336,7 +359,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -352,7 +375,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -648,48 +671,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C52200B-3B0C-4F93-BC6C-7CAE122E49C2}">
-  <dimension ref="A1:AS1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AT1"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" customWidth="1"/>
-    <col min="11" max="11" width="14.109375" customWidth="1"/>
-    <col min="12" max="13" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.33203125" customWidth="1"/>
-    <col min="15" max="15" width="20.5546875" customWidth="1"/>
-    <col min="16" max="16" width="14.88671875" customWidth="1"/>
-    <col min="17" max="17" width="32.44140625" customWidth="1"/>
-    <col min="18" max="18" width="19.6640625" customWidth="1"/>
-    <col min="19" max="19" width="23.88671875" customWidth="1"/>
-    <col min="20" max="22" width="27.109375" customWidth="1"/>
-    <col min="23" max="23" width="16.88671875" customWidth="1"/>
-    <col min="24" max="24" width="14.6640625" customWidth="1"/>
-    <col min="25" max="26" width="16.6640625" customWidth="1"/>
-    <col min="27" max="27" width="19.44140625" customWidth="1"/>
-    <col min="28" max="28" width="14.6640625" customWidth="1"/>
-    <col min="29" max="29" width="14.33203125" customWidth="1"/>
-    <col min="30" max="30" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.375" customWidth="1"/>
+    <col min="4" max="4" width="10.625" customWidth="1"/>
+    <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="6" max="6" width="16.125" customWidth="1"/>
+    <col min="7" max="7" width="11.875" customWidth="1"/>
+    <col min="11" max="11" width="14.125" customWidth="1"/>
+    <col min="12" max="13" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.375" customWidth="1"/>
+    <col min="15" max="15" width="20.5" customWidth="1"/>
+    <col min="16" max="16" width="14.875" customWidth="1"/>
+    <col min="17" max="17" width="32.5" customWidth="1"/>
+    <col min="18" max="18" width="19.625" customWidth="1"/>
+    <col min="19" max="19" width="23.875" customWidth="1"/>
+    <col min="20" max="22" width="27.125" customWidth="1"/>
+    <col min="23" max="23" width="16.875" customWidth="1"/>
+    <col min="24" max="24" width="14.625" customWidth="1"/>
+    <col min="25" max="26" width="16.625" customWidth="1"/>
+    <col min="27" max="27" width="19.5" customWidth="1"/>
+    <col min="28" max="28" width="14.625" customWidth="1"/>
+    <col min="29" max="29" width="14.375" customWidth="1"/>
+    <col min="30" max="30" width="23.375" customWidth="1"/>
     <col min="31" max="31" width="14" customWidth="1"/>
-    <col min="32" max="32" width="13.88671875" customWidth="1"/>
-    <col min="33" max="33" width="17.5546875" customWidth="1"/>
-    <col min="34" max="34" width="18.109375" customWidth="1"/>
+    <col min="32" max="32" width="13.875" customWidth="1"/>
+    <col min="33" max="33" width="17.5" customWidth="1"/>
+    <col min="34" max="34" width="18.125" customWidth="1"/>
     <col min="35" max="35" width="20" customWidth="1"/>
-    <col min="36" max="36" width="29.109375" customWidth="1"/>
-    <col min="37" max="37" width="21.88671875" customWidth="1"/>
-    <col min="38" max="38" width="22.5546875" customWidth="1"/>
-    <col min="39" max="39" width="20.109375" customWidth="1"/>
-    <col min="40" max="40" width="21.88671875" customWidth="1"/>
-    <col min="41" max="41" width="22.5546875" customWidth="1"/>
+    <col min="36" max="36" width="29.125" customWidth="1"/>
+    <col min="37" max="37" width="21.875" customWidth="1"/>
+    <col min="38" max="38" width="22.5" customWidth="1"/>
+    <col min="39" max="39" width="20.125" customWidth="1"/>
+    <col min="40" max="40" width="21.875" customWidth="1"/>
+    <col min="41" max="41" width="22.5" customWidth="1"/>
     <col min="42" max="42" width="22" customWidth="1"/>
-    <col min="43" max="43" width="21.88671875" customWidth="1"/>
-    <col min="44" max="44" width="22.5546875" customWidth="1"/>
-    <col min="45" max="45" width="23.33203125" customWidth="1"/>
+    <col min="43" max="43" width="21.875" customWidth="1"/>
+    <col min="44" max="45" width="22.5" customWidth="1"/>
+    <col min="46" max="46" width="23.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:46" s="6" customFormat="1">
       <c r="A1" s="6" t="s">
         <v>52</v>
       </c>
@@ -823,10 +846,14 @@
         <v>61</v>
       </c>
       <c r="AS1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AT1" s="3" t="s">
         <v>56</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -835,19 +862,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD4DBF4-FEF1-4385-BAD9-BD07A4FA541B}">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="15.88671875" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" customWidth="1"/>
-    <col min="5" max="5" width="20.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" customWidth="1"/>
-    <col min="8" max="8" width="42.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.375" customWidth="1"/>
+    <col min="2" max="2" width="15.875" customWidth="1"/>
+    <col min="3" max="3" width="14.625" customWidth="1"/>
+    <col min="4" max="4" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="20.875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.875" customWidth="1"/>
+    <col min="8" max="8" width="42.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18">
       <c r="A1" s="3" t="s">
         <v>51</v>
       </c>
@@ -874,6 +901,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -882,24 +910,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1A9004E-0524-4CCC-A26D-ED41880F2076}">
   <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" customWidth="1"/>
-    <col min="4" max="4" width="25.88671875" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="6" max="7" width="14.44140625" customWidth="1"/>
-    <col min="8" max="8" width="22.88671875" customWidth="1"/>
-    <col min="9" max="10" width="17.6640625" customWidth="1"/>
-    <col min="11" max="11" width="13.5546875" customWidth="1"/>
-    <col min="12" max="12" width="18.88671875" customWidth="1"/>
-    <col min="13" max="13" width="19.44140625" customWidth="1"/>
-    <col min="14" max="14" width="19.6640625" customWidth="1"/>
-    <col min="15" max="15" width="20.88671875" customWidth="1"/>
+    <col min="1" max="1" width="11.5" customWidth="1"/>
+    <col min="2" max="2" width="17.625" customWidth="1"/>
+    <col min="3" max="3" width="20.375" customWidth="1"/>
+    <col min="4" max="4" width="25.875" customWidth="1"/>
+    <col min="5" max="5" width="12.625" customWidth="1"/>
+    <col min="6" max="7" width="14.5" customWidth="1"/>
+    <col min="8" max="8" width="22.875" customWidth="1"/>
+    <col min="9" max="10" width="17.625" customWidth="1"/>
+    <col min="11" max="11" width="13.5" customWidth="1"/>
+    <col min="12" max="12" width="18.875" customWidth="1"/>
+    <col min="13" max="13" width="19.5" customWidth="1"/>
+    <col min="14" max="14" width="19.625" customWidth="1"/>
+    <col min="15" max="15" width="20.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15">
       <c r="A1" s="3" t="s">
         <v>51</v>
       </c>
@@ -947,6 +975,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -955,19 +984,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AAC19D1-83E1-40A1-A742-B0FE561C9C0F}">
   <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20.33203125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" customWidth="1"/>
-    <col min="5" max="5" width="28.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="12.625" customWidth="1"/>
+    <col min="4" max="4" width="17.5" customWidth="1"/>
+    <col min="5" max="5" width="28.125" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
     <col min="7" max="7" width="21" customWidth="1"/>
-    <col min="8" max="8" width="42.88671875" customWidth="1"/>
+    <col min="8" max="8" width="42.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" s="3" t="s">
         <v>51</v>
       </c>
@@ -997,6 +1026,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1005,25 +1035,25 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{644DDB6A-FFA4-49B3-B3EB-E6F6582E54C5}">
   <dimension ref="A1:AV1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="21" max="22" width="28.6640625" customWidth="1"/>
-    <col min="29" max="30" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="34" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="18.6640625" customWidth="1"/>
-    <col min="37" max="37" width="19.109375" customWidth="1"/>
-    <col min="38" max="38" width="18.44140625" customWidth="1"/>
-    <col min="39" max="39" width="14.109375" customWidth="1"/>
-    <col min="40" max="40" width="22.88671875" customWidth="1"/>
-    <col min="41" max="41" width="13.109375" customWidth="1"/>
+    <col min="21" max="22" width="28.625" customWidth="1"/>
+    <col min="29" max="30" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="18.625" customWidth="1"/>
+    <col min="37" max="37" width="19.125" customWidth="1"/>
+    <col min="38" max="38" width="18.5" customWidth="1"/>
+    <col min="39" max="39" width="14.125" customWidth="1"/>
+    <col min="40" max="40" width="22.875" customWidth="1"/>
+    <col min="41" max="41" width="13.125" customWidth="1"/>
     <col min="43" max="43" width="43" customWidth="1"/>
-    <col min="44" max="44" width="17.44140625" customWidth="1"/>
-    <col min="45" max="45" width="19.33203125" customWidth="1"/>
-    <col min="46" max="46" width="21.6640625" customWidth="1"/>
-    <col min="47" max="47" width="24.88671875" customWidth="1"/>
+    <col min="44" max="44" width="17.5" customWidth="1"/>
+    <col min="45" max="45" width="19.375" customWidth="1"/>
+    <col min="46" max="46" width="21.625" customWidth="1"/>
+    <col min="47" max="47" width="24.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="6" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:48" s="6" customFormat="1" ht="18">
       <c r="A1" s="6" t="s">
         <v>52</v>
       </c>
@@ -1170,6 +1200,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>